<commit_message>
Expand sample data with backend and DevOps roles
Adds two more jobs and five more candidates so the demo covers
backend, DevOps, full-stack, and junior profiles, not just data
science and frontend. Regenerates ranked outputs and cached
embeddings to match.
</commit_message>
<xml_diff>
--- a/data/outputs/ranked_output.xlsx
+++ b/data/outputs/ranked_output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>83.26000000000001</v>
+        <v>83.45</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -481,7 +481,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>61.01</v>
+        <v>61.09</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -497,18 +497,18 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C004</t>
+          <t>C009</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>45.49</v>
+        <v>60.27</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Candidate C004 is a moderate fit because they match 2/5 required skills and have 2 years of experience, below the 3-year minimum. Project experience mentions Machine Learning.</t>
+          <t>Candidate C009 is a moderate fit because they match 4/5 required skills and have 1 years of experience, below the 3-year minimum. Projects are listed, but no direct job-skill evidence was detected.</t>
         </is>
       </c>
     </row>
@@ -520,18 +520,18 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>C005</t>
+          <t>C004</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>44.77</v>
+        <v>45.41</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Candidate C005 is a limited fit because they match 1/5 required skills and have 5 years of experience for the 3-6 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+          <t>Candidate C004 is a moderate fit because they match 2/5 required skills and have 2 years of experience, below the 3-year minimum. Project experience mentions Machine Learning.</t>
         </is>
       </c>
     </row>
@@ -543,133 +543,823 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C005</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>25.24</v>
+        <v>44.99</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Candidate C003 is a limited fit because they match 0/5 required skills and have 4 years of experience for the 3-6 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+          <t>Candidate C005 is a limited fit because they match 1/5 required skills and have 5 years of experience for the 3-6 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>J002</t>
+          <t>J001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C006</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
-        <v>83.83</v>
+        <v>36.6</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Candidate C003 is a strong fit because they match 4/4 required skills and have 4 years of experience for the 2-5 year role range. Project experience mentions React, Node.js.</t>
+          <t>Candidate C006 is a limited fit because they match 1/5 required skills and have 3 years of experience for the 3-6 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>J002</t>
+          <t>J001</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C010</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>24.82</v>
+        <v>35.06</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Candidate C001 is a limited fit because they match 0/4 required skills and have 4 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+          <t>Candidate C010 is a limited fit because they match 1/5 required skills and have 6 years of experience for the 3-6 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>J002</t>
+          <t>J001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C008</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>23.62</v>
+        <v>32.7</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Candidate C002 is a limited fit because they match 0/4 required skills and have 3 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+          <t>Candidate C008 is a limited fit because they match 1/5 required skills and have 3 years of experience for the 3-6 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>J002</t>
+          <t>J001</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C005</t>
+          <t>C007</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D10" t="n">
-        <v>21.76</v>
+        <v>28.45</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Candidate C005 is a limited fit because they match 0/4 required skills and have 5 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+          <t>Candidate C007 is a limited fit because they match 0/5 required skills and have 5 years of experience for the 3-6 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>J001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>C003</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="n">
+        <v>25.24</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Candidate C003 is a limited fit because they match 0/5 required skills and have 4 years of experience for the 3-6 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>J002</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>C003</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>83.61</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Candidate C003 is a strong fit because they match 4/4 required skills and have 4 years of experience for the 2-5 year role range. Project experience mentions React, Node.js.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>J002</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>C008</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>79.56999999999999</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Candidate C008 is a strong fit because they match 4/4 required skills and have 3 years of experience for the 2-5 year role range. Project experience mentions React, Node.js.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>J002</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>C006</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>35.21</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Candidate C006 is a limited fit because they match 0/4 required skills and have 3 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>J002</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>C007</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>29.87</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Candidate C007 is a limited fit because they match 0/4 required skills and have 5 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>J002</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>C010</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>28.96</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Candidate C010 is a limited fit because they match 0/4 required skills and have 6 years of experience, above the 5-year maximum. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>J002</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="n">
+        <v>24.82</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Candidate C001 is a limited fit because they match 0/4 required skills and have 4 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>J002</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" t="n">
+        <v>23.62</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Candidate C002 is a limited fit because they match 0/4 required skills and have 3 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>J002</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C005</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>21.76</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Candidate C005 is a limited fit because they match 0/4 required skills and have 5 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>J002</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>C004</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C20" t="n">
+        <v>9</v>
+      </c>
+      <c r="D20" t="n">
+        <v>21.58</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Candidate C004 is a limited fit because they match 0/4 required skills and have 2 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>J002</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>C009</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" t="n">
+        <v>14.64</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Candidate C009 is a limited fit because they match 0/4 required skills and have 1 years of experience, below the 2-year minimum. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>C006</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>85.34999999999999</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Candidate C006 is a strong fit because they match 4/4 required skills and have 3 years of experience for the 2-5 year role range. Project experience mentions rest apis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>C008</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>45.27</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Candidate C008 is a moderate fit because they match 1/4 required skills and have 3 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>C010</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>41.96</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Candidate C010 is a limited fit because they match 1/4 required skills and have 6 years of experience, above the 5-year maximum. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Candidate C001 is a limited fit because they match 1/4 required skills and have 4 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
         <v>5</v>
       </c>
-      <c r="D11" t="n">
-        <v>21.68</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Candidate C004 is a limited fit because they match 0/4 required skills and have 2 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+      <c r="D26" t="n">
+        <v>35.95</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Candidate C002 is a limited fit because they match 1/4 required skills and have 3 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C003</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" t="n">
+        <v>34.82</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Candidate C003 is a limited fit because they match 0/4 required skills and have 4 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>C007</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>31.58</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Candidate C007 is a limited fit because they match 0/4 required skills and have 5 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>C004</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" t="n">
+        <v>31.39</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Candidate C004 is a limited fit because they match 1/4 required skills and have 2 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>C009</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>9</v>
+      </c>
+      <c r="D30" t="n">
+        <v>28.27</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Candidate C009 is a limited fit because they match 1/4 required skills and have 1 years of experience, below the 2-year minimum. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>J003</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>C005</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" t="n">
+        <v>26.07</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Candidate C005 is a limited fit because they match 0/4 required skills and have 5 years of experience for the 2-5 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>C007</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>85.88</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Candidate C007 is a strong fit because they match 5/5 required skills and have 5 years of experience for the 3-7 year role range. Project experience mentions Kubernetes, ci/cd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>C010</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Candidate C010 is a moderate fit because they match 4/5 required skills and have 6 years of experience for the 3-7 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>C008</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>39.65</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Candidate C008 is a limited fit because they match 1/5 required skills and have 3 years of experience for the 3-7 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>C006</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>4</v>
+      </c>
+      <c r="D35" t="n">
+        <v>36.17</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Candidate C006 is a limited fit because they match 1/5 required skills and have 3 years of experience for the 3-7 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>C003</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>5</v>
+      </c>
+      <c r="D36" t="n">
+        <v>35.32</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Candidate C003 is a limited fit because they match 1/5 required skills and have 4 years of experience for the 3-7 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>6</v>
+      </c>
+      <c r="D37" t="n">
+        <v>32.07</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Candidate C001 is a limited fit because they match 1/5 required skills and have 4 years of experience for the 3-7 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>C005</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>7</v>
+      </c>
+      <c r="D38" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Candidate C005 is a limited fit because they match 0/5 required skills and have 5 years of experience for the 3-7 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D39" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Candidate C002 is a limited fit because they match 0/5 required skills and have 3 years of experience for the 3-7 year role range. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>C004</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>9</v>
+      </c>
+      <c r="D40" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Candidate C004 is a limited fit because they match 0/5 required skills and have 2 years of experience, below the 3-year minimum. Projects are listed, but no direct job-skill evidence was detected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>J004</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>C009</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Candidate C009 is a limited fit because they match 0/5 required skills and have 1 years of experience, below the 3-year minimum. Projects are listed, but no direct job-skill evidence was detected.</t>
         </is>
       </c>
     </row>

</xml_diff>